<commit_message>
Add exercise materials and tools for hands-on workshop on documentation in the AI era
- Introduced new directory `examples/business-trip/exercise/` containing exercise materials for the business trip application system, including design documents and templates.
- Added `requirements.template.md` to guide users in creating requirements documents.
- Created `README.md` in the exercise directory to explain the purpose and structure of the materials.
- Implemented `tools/exercise-dist/` to build a distribution subset for workshop participants, excluding answers and providing necessary files.
- Added `build.py` script to automate the creation of the distribution package.
- Updated existing documentation to reference new exercise materials and correct links.
</commit_message>
<xml_diff>
--- a/examples/business-trip/traditional-design/システム機能設計書(画面)_BTS04_最終承認.xlsx
+++ b/examples/business-trip/traditional-design/システム機能設計書(画面)_BTS04_最終承認.xlsx
@@ -9516,18 +9516,18 @@
       <c r="F114" s="100" t="n"/>
       <c r="G114" s="121" t="inlineStr">
         <is>
-          <t>申請ID</t>
+          <t>レコード区分</t>
         </is>
       </c>
       <c r="K114" s="121" t="n">
         <v>1</v>
       </c>
       <c r="N114" s="121" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="Q114" s="121" t="inlineStr">
         <is>
-          <t>application_id。半角英数字16桁。左詰めとし、残りは半角空白で埋める。</t>
+          <t>明細レコードを表す固定値 '2'。</t>
         </is>
       </c>
       <c r="AJ114" s="93" t="n"/>
@@ -9536,58 +9536,58 @@
       <c r="F115" s="100" t="n"/>
       <c r="G115" s="121" t="inlineStr">
         <is>
-          <t>社員番号</t>
+          <t>申請ID</t>
         </is>
       </c>
       <c r="K115" s="121" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="N115" s="121" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="Q115" s="121" t="inlineStr">
         <is>
-          <t>applicant_id。半角英数字10桁。</t>
+          <t>application_id。半角英数字16桁。左詰めとし、残りは半角空白で埋める。</t>
         </is>
       </c>
       <c r="AJ115" s="93" t="n"/>
     </row>
-    <row r="116" ht="30" customHeight="1" s="91">
+    <row r="116" ht="16" customHeight="1" s="91">
       <c r="F116" s="100" t="n"/>
       <c r="G116" s="121" t="inlineStr">
         <is>
-          <t>精算額</t>
+          <t>申請者社員番号</t>
         </is>
       </c>
       <c r="K116" s="121" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="N116" s="121" t="n">
         <v>10</v>
       </c>
       <c r="Q116" s="121" t="inlineStr">
         <is>
-          <t>(4)で算出した精算額。ゾーン10進10桁、右詰めゼロ埋め（0円の場合も 0000000000 を出力する）。</t>
+          <t>applicant_id。半角英数字10桁。</t>
         </is>
       </c>
       <c r="AJ116" s="93" t="n"/>
     </row>
-    <row r="117" ht="16" customHeight="1" s="91">
+    <row r="117" ht="30" customHeight="1" s="91">
       <c r="F117" s="100" t="n"/>
       <c r="G117" s="121" t="inlineStr">
         <is>
-          <t>費用負担区分</t>
+          <t>精算額</t>
         </is>
       </c>
       <c r="K117" s="121" t="n">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="N117" s="121" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="Q117" s="121" t="inlineStr">
         <is>
-          <t>cost_bearing。1桁（1:自社負担 / 2:先方負担）。</t>
+          <t>(4)で算出した精算額。半角数字9桁、右詰め前ゼロ埋め（0円の場合も 000000000 を出力する）。</t>
         </is>
       </c>
       <c r="AJ117" s="93" t="n"/>
@@ -9596,142 +9596,104 @@
       <c r="F118" s="100" t="n"/>
       <c r="G118" s="121" t="inlineStr">
         <is>
-          <t>最終承認日時</t>
+          <t>費用負担区分</t>
         </is>
       </c>
       <c r="K118" s="121" t="n">
         <v>38</v>
       </c>
       <c r="N118" s="121" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="Q118" s="121" t="inlineStr">
         <is>
-          <t>finalized_at。YYYYMMDDHHMMSS形式の14桁。</t>
+          <t>cost_bearing。2桁（01:自社負担 / 02:先方負担）。</t>
         </is>
       </c>
       <c r="AJ118" s="93" t="n"/>
     </row>
-    <row r="119" ht="30" customHeight="1" s="91">
-      <c r="F119" s="121" t="inlineStr">
-        <is>
-          <t>ヘッダレコードにはレコード種別'H'とファイル作成日時を、トレーラレコードにはレコード種別'T'・データレコード件数・精算額合計を出力する。</t>
+    <row r="119" ht="16" customHeight="1" s="91">
+      <c r="F119" s="100" t="n"/>
+      <c r="G119" s="121" t="inlineStr">
+        <is>
+          <t>最終承認日</t>
+        </is>
+      </c>
+      <c r="K119" s="121" t="n">
+        <v>40</v>
+      </c>
+      <c r="N119" s="121" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q119" s="121" t="inlineStr">
+        <is>
+          <t>finalized_at の日付部。YYYYMMDD形式の8桁。</t>
         </is>
       </c>
       <c r="AJ119" s="93" t="n"/>
     </row>
     <row r="120" ht="16" customHeight="1" s="91">
-      <c r="E120" s="121" t="inlineStr">
+      <c r="F120" s="100" t="n"/>
+      <c r="G120" s="121" t="inlineStr">
+        <is>
+          <t>部門コード</t>
+        </is>
+      </c>
+      <c r="K120" s="121" t="n">
+        <v>48</v>
+      </c>
+      <c r="N120" s="121" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q120" s="121" t="inlineStr">
+        <is>
+          <t>申請者の所属部門コード（BT_EMPLOYEE.department_code）。</t>
+        </is>
+      </c>
+      <c r="AJ120" s="93" t="n"/>
+    </row>
+    <row r="121" ht="16" customHeight="1" s="91">
+      <c r="F121" s="100" t="n"/>
+      <c r="G121" s="121" t="inlineStr">
+        <is>
+          <t>FILLER</t>
+        </is>
+      </c>
+      <c r="K121" s="121" t="n">
+        <v>78</v>
+      </c>
+      <c r="N121" s="121" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q121" s="121" t="inlineStr">
+        <is>
+          <t>半角空白で埋める。</t>
+        </is>
+      </c>
+      <c r="AJ121" s="93" t="n"/>
+    </row>
+    <row r="122" ht="30" customHeight="1" s="91">
+      <c r="F122" s="121" t="inlineStr">
+        <is>
+          <t>ヘッダレコードにはレコード区分'1'・ファイルID・作成日を、トレーラレコードにはレコード区分'9'・明細件数・精算額合計を出力する。レコードの詳細レイアウトは外部インタフェース設計書(IBT01)による。</t>
+        </is>
+      </c>
+      <c r="AJ122" s="93" t="n"/>
+    </row>
+    <row r="123" ht="16" customHeight="1" s="91">
+      <c r="E123" s="121" t="inlineStr">
         <is>
           <t>(6) 表示処理</t>
         </is>
       </c>
-      <c r="AJ120" s="93" t="n"/>
-    </row>
-    <row r="121" ht="16" customHeight="1" s="91">
-      <c r="F121" s="121" t="inlineStr">
+      <c r="AJ123" s="93" t="n"/>
+    </row>
+    <row r="124" ht="16" customHeight="1" s="91">
+      <c r="F124" s="121" t="inlineStr">
         <is>
           <t>経理連携完了メッセージ（MSG10003）を表示し、出張申請一覧画面（WBT0501）へ遷移する。</t>
         </is>
       </c>
-      <c r="AJ121" s="93" t="n"/>
-    </row>
-    <row r="122">
-      <c r="F122" s="100" t="n"/>
-      <c r="G122" s="100" t="n"/>
-      <c r="H122" s="100" t="n"/>
-      <c r="I122" s="100" t="n"/>
-      <c r="J122" s="100" t="n"/>
-      <c r="K122" s="100" t="n"/>
-      <c r="L122" s="100" t="n"/>
-      <c r="M122" s="100" t="n"/>
-      <c r="N122" s="100" t="n"/>
-      <c r="O122" s="100" t="n"/>
-      <c r="P122" s="100" t="n"/>
-      <c r="Q122" s="100" t="n"/>
-      <c r="R122" s="100" t="n"/>
-      <c r="S122" s="100" t="n"/>
-      <c r="T122" s="100" t="n"/>
-      <c r="U122" s="100" t="n"/>
-      <c r="V122" s="100" t="n"/>
-      <c r="W122" s="100" t="n"/>
-      <c r="X122" s="100" t="n"/>
-      <c r="Y122" s="100" t="n"/>
-      <c r="Z122" s="100" t="n"/>
-      <c r="AA122" s="100" t="n"/>
-      <c r="AB122" s="100" t="n"/>
-      <c r="AC122" s="100" t="n"/>
-      <c r="AD122" s="100" t="n"/>
-      <c r="AE122" s="100" t="n"/>
-      <c r="AF122" s="100" t="n"/>
-      <c r="AG122" s="100" t="n"/>
-      <c r="AH122" s="100" t="n"/>
-      <c r="AI122" s="100" t="n"/>
-      <c r="AJ122" s="93" t="n"/>
-    </row>
-    <row r="123">
-      <c r="F123" s="100" t="n"/>
-      <c r="G123" s="100" t="n"/>
-      <c r="H123" s="100" t="n"/>
-      <c r="I123" s="100" t="n"/>
-      <c r="J123" s="100" t="n"/>
-      <c r="K123" s="100" t="n"/>
-      <c r="L123" s="100" t="n"/>
-      <c r="M123" s="100" t="n"/>
-      <c r="N123" s="100" t="n"/>
-      <c r="O123" s="100" t="n"/>
-      <c r="P123" s="100" t="n"/>
-      <c r="Q123" s="100" t="n"/>
-      <c r="R123" s="100" t="n"/>
-      <c r="S123" s="100" t="n"/>
-      <c r="T123" s="100" t="n"/>
-      <c r="U123" s="100" t="n"/>
-      <c r="V123" s="100" t="n"/>
-      <c r="W123" s="100" t="n"/>
-      <c r="X123" s="100" t="n"/>
-      <c r="Y123" s="100" t="n"/>
-      <c r="Z123" s="100" t="n"/>
-      <c r="AA123" s="100" t="n"/>
-      <c r="AB123" s="100" t="n"/>
-      <c r="AC123" s="100" t="n"/>
-      <c r="AD123" s="100" t="n"/>
-      <c r="AE123" s="100" t="n"/>
-      <c r="AF123" s="100" t="n"/>
-      <c r="AG123" s="100" t="n"/>
-      <c r="AH123" s="100" t="n"/>
-      <c r="AI123" s="100" t="n"/>
-      <c r="AJ123" s="93" t="n"/>
-    </row>
-    <row r="124">
-      <c r="F124" s="100" t="n"/>
-      <c r="G124" s="100" t="n"/>
-      <c r="H124" s="100" t="n"/>
-      <c r="I124" s="100" t="n"/>
-      <c r="J124" s="100" t="n"/>
-      <c r="K124" s="100" t="n"/>
-      <c r="L124" s="100" t="n"/>
-      <c r="M124" s="100" t="n"/>
-      <c r="N124" s="100" t="n"/>
-      <c r="O124" s="100" t="n"/>
-      <c r="P124" s="100" t="n"/>
-      <c r="Q124" s="100" t="n"/>
-      <c r="R124" s="100" t="n"/>
-      <c r="S124" s="100" t="n"/>
-      <c r="T124" s="100" t="n"/>
-      <c r="U124" s="100" t="n"/>
-      <c r="V124" s="100" t="n"/>
-      <c r="W124" s="100" t="n"/>
-      <c r="X124" s="100" t="n"/>
-      <c r="Y124" s="100" t="n"/>
-      <c r="Z124" s="100" t="n"/>
-      <c r="AA124" s="100" t="n"/>
-      <c r="AB124" s="100" t="n"/>
-      <c r="AC124" s="100" t="n"/>
-      <c r="AD124" s="100" t="n"/>
-      <c r="AE124" s="100" t="n"/>
-      <c r="AF124" s="100" t="n"/>
-      <c r="AG124" s="100" t="n"/>
-      <c r="AI124" s="100" t="n"/>
       <c r="AJ124" s="93" t="n"/>
     </row>
     <row r="125">
@@ -10140,14 +10102,16 @@
     <row r="168"/>
     <row r="169"/>
   </sheetData>
-  <mergeCells count="253">
+  <mergeCells count="265">
     <mergeCell ref="T77:U77"/>
     <mergeCell ref="V73:AH74"/>
+    <mergeCell ref="K119:M119"/>
     <mergeCell ref="AE69:AH69"/>
     <mergeCell ref="AE84:AH84"/>
     <mergeCell ref="F67:I67"/>
     <mergeCell ref="J56:M56"/>
     <mergeCell ref="S1:Z3"/>
+    <mergeCell ref="G119:J119"/>
     <mergeCell ref="AL63:AO63"/>
     <mergeCell ref="F52:AD52"/>
     <mergeCell ref="U132:AA132"/>
@@ -10155,6 +10119,8 @@
     <mergeCell ref="E77:J77"/>
     <mergeCell ref="T78:U78"/>
     <mergeCell ref="D99:AI99"/>
+    <mergeCell ref="Q120:AI120"/>
+    <mergeCell ref="K120:M120"/>
     <mergeCell ref="V63:Z63"/>
     <mergeCell ref="F109:AI109"/>
     <mergeCell ref="AB134:AI134"/>
@@ -10174,12 +10140,14 @@
     <mergeCell ref="F59:I59"/>
     <mergeCell ref="N57:U57"/>
     <mergeCell ref="D73:D74"/>
+    <mergeCell ref="K121:M121"/>
     <mergeCell ref="K76:N76"/>
     <mergeCell ref="AB129:AI130"/>
     <mergeCell ref="V66:Z66"/>
     <mergeCell ref="D130:K130"/>
     <mergeCell ref="AA2:AB2"/>
     <mergeCell ref="AA53:AC54"/>
+    <mergeCell ref="G121:J121"/>
     <mergeCell ref="AE82:AH82"/>
     <mergeCell ref="O1:R3"/>
     <mergeCell ref="Z84:AD84"/>
@@ -10190,6 +10158,7 @@
     <mergeCell ref="G114:J114"/>
     <mergeCell ref="AL62:AO62"/>
     <mergeCell ref="Q114:AI114"/>
+    <mergeCell ref="F124:AI124"/>
     <mergeCell ref="J53:M54"/>
     <mergeCell ref="AG2:AI2"/>
     <mergeCell ref="V61:Z61"/>
@@ -10239,6 +10208,7 @@
     <mergeCell ref="J68:M68"/>
     <mergeCell ref="N113:P113"/>
     <mergeCell ref="AE62:AH62"/>
+    <mergeCell ref="Q121:AI121"/>
     <mergeCell ref="V77:AH77"/>
     <mergeCell ref="T75:U75"/>
     <mergeCell ref="AD53:AD54"/>
@@ -10278,6 +10248,7 @@
     <mergeCell ref="F104:AI104"/>
     <mergeCell ref="AB132:AI132"/>
     <mergeCell ref="N66:U66"/>
+    <mergeCell ref="N120:P120"/>
     <mergeCell ref="AA68:AC68"/>
     <mergeCell ref="J61:M61"/>
     <mergeCell ref="E46:M46"/>
@@ -10286,6 +10257,7 @@
     <mergeCell ref="F64:I64"/>
     <mergeCell ref="E100:AI100"/>
     <mergeCell ref="F106:AI106"/>
+    <mergeCell ref="N119:P119"/>
     <mergeCell ref="AL53:AO54"/>
     <mergeCell ref="AA66:AC66"/>
     <mergeCell ref="N68:U68"/>
@@ -10326,13 +10298,13 @@
     <mergeCell ref="K84:Q84"/>
     <mergeCell ref="AL57:AO57"/>
     <mergeCell ref="G118:J118"/>
-    <mergeCell ref="F119:AI119"/>
     <mergeCell ref="F66:I66"/>
     <mergeCell ref="V46:AC46"/>
     <mergeCell ref="V57:Z57"/>
     <mergeCell ref="AA58:AC58"/>
     <mergeCell ref="F103:AI103"/>
     <mergeCell ref="U130:AA130"/>
+    <mergeCell ref="N121:P121"/>
     <mergeCell ref="V47:AC47"/>
     <mergeCell ref="N115:P115"/>
     <mergeCell ref="N46:P46"/>
@@ -10347,13 +10319,14 @@
     <mergeCell ref="AL58:AO58"/>
     <mergeCell ref="E78:J78"/>
     <mergeCell ref="F95:AI95"/>
+    <mergeCell ref="Q119:AI119"/>
     <mergeCell ref="E110:AI110"/>
     <mergeCell ref="N116:P116"/>
     <mergeCell ref="AA63:AC63"/>
     <mergeCell ref="N56:U56"/>
-    <mergeCell ref="E120:AI120"/>
     <mergeCell ref="K115:M115"/>
     <mergeCell ref="AL60:AO60"/>
+    <mergeCell ref="F122:AI122"/>
     <mergeCell ref="F97:AI97"/>
     <mergeCell ref="E45:M45"/>
     <mergeCell ref="AL69:AO69"/>
@@ -10367,7 +10340,7 @@
     <mergeCell ref="F65:I65"/>
     <mergeCell ref="E73:J74"/>
     <mergeCell ref="R83:Y83"/>
-    <mergeCell ref="F121:AI121"/>
+    <mergeCell ref="G120:J120"/>
     <mergeCell ref="Q116:AI116"/>
     <mergeCell ref="AL61:AO61"/>
     <mergeCell ref="AE58:AH58"/>
@@ -10377,6 +10350,7 @@
     <mergeCell ref="V78:AH78"/>
     <mergeCell ref="N59:U59"/>
     <mergeCell ref="D129:AA129"/>
+    <mergeCell ref="E123:AI123"/>
     <mergeCell ref="N60:U60"/>
     <mergeCell ref="AA3:AB3"/>
     <mergeCell ref="K75:N75"/>

</xml_diff>